<commit_message>
update: 2026-09-10 周巡查表 Excel 补入周三 9 场所（112 行 / 365 项）
</commit_message>
<xml_diff>
--- a/weeks/2026-09-10/巡查表.xlsx
+++ b/weeks/2026-09-10/巡查表.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:Z105"/>
+  <dimension ref="A2:Z114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -13181,6 +13181,559 @@
       <c r="Z105" t="inlineStr">
         <is>
           <t>否</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>城中村</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>马坑</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>龙岗区</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>南澳街道</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>广东省深圳市龙岗区南澳街道南澳派出所辖区工作点大鹏新区</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>1.6: 设置洗手设施。（2分） (-1)
+1.13: 收集容器外壁及内桶保持干净整洁，避免陈旧性脏污，收集容器内无积水。（6分） (-3)
+1.14: 各类垃圾及时清运，投放点及其周围环境干净整洁，没有垃圾满溢、暴露垃圾、杂物堆放、严重积水或明显异味等问题。（6分） (-2)
+1.17: 转运桶应在黄线划定区域内摆放整齐并保持全天关闭（作业状态除外），禁止罩外摆桶供居民投放。（6分） (-2)
+2.2: 设置消防设施，使用功能正常，取用方便。（2分） (-2)
+2.3: 各类垃圾及时清运。（2分） (-2)</t>
+        </is>
+      </c>
+      <c r="O106" s="4" t="inlineStr">
+        <is>
+          <t>查看证据(6项/6张)</t>
+        </is>
+      </c>
+      <c r="P106" t="n">
+        <v>88</v>
+      </c>
+      <c r="T106" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="U106" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="V106" t="inlineStr">
+        <is>
+          <t>2026-09-16 14:01:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>住宅小区</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>南澳湾花园</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>龙岗区</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>南澳街道</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>广东省深圳市龙岗区南澳街道南澳湾花园</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>2.2: 设置消防设施，使用功能正常，取用方便。（2分） (-2)
+2.3: 各类垃圾及时清运。（2分） (-2)</t>
+        </is>
+      </c>
+      <c r="O107" s="4" t="inlineStr">
+        <is>
+          <t>查看证据(2项/2张)</t>
+        </is>
+      </c>
+      <c r="P107" t="n">
+        <v>96</v>
+      </c>
+      <c r="T107" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="U107" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="V107" t="inlineStr">
+        <is>
+          <t>2026-09-16 14:02:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>城中村</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>老街</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>龙岗区</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>南澳街道</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>广东省深圳市龙岗区南澳街道南澳湾花园大鹏新区</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>1.17: 转运桶应在黄线划定区域内摆放整齐并保持全天关闭（作业状态除外），禁止罩外摆桶供居民投放。（6分） (-2)
+2.2: 设置消防设施，使用功能正常，取用方便。（2分） (-2)
+2.3: 各类垃圾及时清运。（2分） (-2)</t>
+        </is>
+      </c>
+      <c r="O108" s="4" t="inlineStr">
+        <is>
+          <t>查看证据(3项/4张)</t>
+        </is>
+      </c>
+      <c r="P108" t="n">
+        <v>94</v>
+      </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="U108" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="V108" t="inlineStr">
+        <is>
+          <t>2026-09-16 14:02:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>城中村</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>风球山小区</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>龙岗区</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>南澳街道</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>广东省深圳市龙岗区南澳街道风球山小区</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>1.17: 转运桶应在黄线划定区域内摆放整齐并保持全天关闭（作业状态除外），禁止罩外摆桶供居民投放。（6分） (-2)
+2.2: 设置消防设施，使用功能正常，取用方便。（2分） (-2)
+2.3: 各类垃圾及时清运。（2分） (-2)</t>
+        </is>
+      </c>
+      <c r="O109" s="4" t="inlineStr">
+        <is>
+          <t>查看证据(3项/3张)</t>
+        </is>
+      </c>
+      <c r="P109" t="n">
+        <v>94</v>
+      </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="U109" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="V109" t="inlineStr">
+        <is>
+          <t>2026-09-16 14:02:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>城中村</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>上企沙</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>龙岗区</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>南澳街道</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>广东省深圳市龙岗区南澳街道上企沙大鹏新区</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>1.17: 转运桶应在黄线划定区域内摆放整齐并保持全天关闭（作业状态除外），禁止罩外摆桶供居民投放。（6分） (-2)</t>
+        </is>
+      </c>
+      <c r="O110" s="4" t="inlineStr">
+        <is>
+          <t>查看证据(1项/1张)</t>
+        </is>
+      </c>
+      <c r="P110" t="n">
+        <v>98</v>
+      </c>
+      <c r="T110" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="U110" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="V110" t="inlineStr">
+        <is>
+          <t>2026-09-16 14:02:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>住宅小区</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>山海名苑</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>龙岗区</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>南澳街道</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>广东省深圳市龙岗区南澳街道山海名苑</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>1.17: 转运桶应在黄线划定区域内摆放整齐并保持全天关闭（作业状态除外），禁止罩外摆桶供居民投放。（6分） (-4)</t>
+        </is>
+      </c>
+      <c r="O111" s="4" t="inlineStr">
+        <is>
+          <t>查看证据(1项/2张)</t>
+        </is>
+      </c>
+      <c r="P111" t="n">
+        <v>96</v>
+      </c>
+      <c r="T111" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="U111" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="V111" t="inlineStr">
+        <is>
+          <t>2026-09-16 14:02:22</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>城中村</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>下企沙</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>龙岗区</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>南澳街道</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>广东省深圳市龙岗区南澳街道企沙下路大鹏新区</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>1.17: 转运桶应在黄线划定区域内摆放整齐并保持全天关闭（作业状态除外），禁止罩外摆桶供居民投放。（6分） (-2)</t>
+        </is>
+      </c>
+      <c r="O112" s="4" t="inlineStr">
+        <is>
+          <t>查看证据(1项/2张)</t>
+        </is>
+      </c>
+      <c r="P112" t="n">
+        <v>98</v>
+      </c>
+      <c r="T112" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="U112" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="V112" t="inlineStr">
+        <is>
+          <t>2026-09-16 14:02:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>住宅小区</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>金地朗悦西区</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>坪山区</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>马峦街道</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>坪山区马峦街道金地朗悦西区3栋集中分类投放点</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>1.5: 分类标志完整、正确、清晰，各类垃圾收集容器外罩和内桶的颜色正确。（4分） (-4)
+1.13: 收集容器外壁及内桶保持干净整洁，避免陈旧性脏污，收集容器内无积水。（4分） (-2)
+2.1: 设置标识牌，外观使用“深i回收”标识，封闭围挡，地面硬底化。（2分） (-2)</t>
+        </is>
+      </c>
+      <c r="O113" s="4" t="inlineStr">
+        <is>
+          <t>查看证据(3项/5张)</t>
+        </is>
+      </c>
+      <c r="P113" t="n">
+        <v>92</v>
+      </c>
+      <c r="T113" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="U113" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="V113" t="inlineStr">
+        <is>
+          <t>2026-09-16 12:11:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>住宅小区</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>金地朗悦东区</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>坪山区</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>马峦街道</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>坪山区马峦街道金地朗悦东区1栋集中分类投放点</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>1.6: 设置洗手设施。（2分） (-1)
+2.1: 设置标识牌，外观使用“深i回收”标识，封闭围挡，地面硬底化。（2分） (-2)</t>
+        </is>
+      </c>
+      <c r="O114" s="4" t="inlineStr">
+        <is>
+          <t>查看证据(2项/3张)</t>
+        </is>
+      </c>
+      <c r="P114" t="n">
+        <v>97</v>
+      </c>
+      <c r="T114" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="U114" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="V114" t="inlineStr">
+        <is>
+          <t>2026-09-16 12:11:47</t>
         </is>
       </c>
     </row>
@@ -13289,6 +13842,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O103" r:id="rId101"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O104" r:id="rId102"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O105" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O106" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O107" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O108" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O109" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O110" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O111" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O112" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O113" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O114" r:id="rId112"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13300,7 +13862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G344"/>
+  <dimension ref="A1:G366"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -23704,7 +24266,11 @@
           <t>-3</t>
         </is>
       </c>
-      <c r="F315" s="6" t="inlineStr"/>
+      <c r="F315" s="6" t="inlineStr">
+        <is>
+          <t>（2）未成组摆放两分类收集容器(-3)（1处问题）</t>
+        </is>
+      </c>
       <c r="G315" s="4" t="inlineStr">
         <is>
           <t>查看证据</t>
@@ -23737,7 +24303,11 @@
           <t>-5</t>
         </is>
       </c>
-      <c r="F316" s="6" t="inlineStr"/>
+      <c r="F316" s="6" t="inlineStr">
+        <is>
+          <t>（2）收集容器缺失(-5)（1处问题）</t>
+        </is>
+      </c>
       <c r="G316" s="4" t="inlineStr">
         <is>
           <t>查看证据</t>
@@ -23770,7 +24340,11 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F317" s="6" t="inlineStr"/>
+      <c r="F317" s="6" t="inlineStr">
+        <is>
+          <t>（2）收集容器缺失</t>
+        </is>
+      </c>
       <c r="G317" s="4" t="inlineStr">
         <is>
           <t>查看证据</t>
@@ -23803,7 +24377,11 @@
           <t>-3</t>
         </is>
       </c>
-      <c r="F318" s="6" t="inlineStr"/>
+      <c r="F318" s="6" t="inlineStr">
+        <is>
+          <t>（2）收集容器标志缺失、错误或模糊不清的。（不强制要求垃圾桶套袋，若套袋的，收集容器应按垃圾类别对应颜色套袋）(-3)（1处问题）</t>
+        </is>
+      </c>
       <c r="G318" s="4" t="inlineStr">
         <is>
           <t>查看证据</t>
@@ -23836,7 +24414,11 @@
           <t>-4</t>
         </is>
       </c>
-      <c r="F319" s="6" t="inlineStr"/>
+      <c r="F319" s="6" t="inlineStr">
+        <is>
+          <t>（2）未按要求张贴垃圾分类宣传海报/指引，或海报内容错误/未更新等(-4)（1处问题）</t>
+        </is>
+      </c>
       <c r="G319" s="4" t="inlineStr">
         <is>
           <t>查看证据</t>
@@ -24663,6 +25245,820 @@
       </c>
       <c r="F344" s="6" t="inlineStr"/>
       <c r="G344" s="4" t="inlineStr">
+        <is>
+          <t>查看证据</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>城中村</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>马坑</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="D345" s="6" t="inlineStr">
+        <is>
+          <t>设置洗手设施。（2分）</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>-1</t>
+        </is>
+      </c>
+      <c r="F345" s="6" t="inlineStr">
+        <is>
+          <t>（3）洗手设施不规范（包括水龙头损坏或明显松动，水龙头不出水，洗手盆堵塞等）(-1)（1处问题）</t>
+        </is>
+      </c>
+      <c r="G345" s="4" t="inlineStr">
+        <is>
+          <t>查看证据</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>城中村</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>马坑</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>1.13</t>
+        </is>
+      </c>
+      <c r="D346" s="6" t="inlineStr">
+        <is>
+          <t>收集容器外壁及内桶保持干净整洁，避免陈旧性脏污，收集容器内无积水。（6分）</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>-3</t>
+        </is>
+      </c>
+      <c r="F346" s="6" t="inlineStr">
+        <is>
+          <t>（2）收集容器外壁、内桶存在明显陈旧性脏污，大片锈迹等(-3)（1处问题）</t>
+        </is>
+      </c>
+      <c r="G346" s="4" t="inlineStr">
+        <is>
+          <t>查看证据</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>城中村</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>马坑</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>1.14</t>
+        </is>
+      </c>
+      <c r="D347" s="6" t="inlineStr">
+        <is>
+          <t>各类垃圾及时清运，投放点及其周围环境干净整洁，没有垃圾满溢、暴露垃圾、杂物堆放、严重积水或明显异味等问题。（6分）</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
+      </c>
+      <c r="F347" s="6" t="inlineStr">
+        <is>
+          <t>（3）环境卫生不整洁（投放点有暴露垃圾、杂物堆放，洗手池严重脏污，地面未硬底化，有明显污水污渍等）(-2)（1处问题）</t>
+        </is>
+      </c>
+      <c r="G347" s="4" t="inlineStr">
+        <is>
+          <t>查看证据</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>城中村</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>马坑</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>1.17</t>
+        </is>
+      </c>
+      <c r="D348" s="6" t="inlineStr">
+        <is>
+          <t>转运桶应在黄线划定区域内摆放整齐并保持全天关闭（作业状态除外），禁止罩外摆桶供居民投放。（6分）</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
+      </c>
+      <c r="F348" s="6" t="inlineStr">
+        <is>
+          <t>（3）监控范围外罩外摆桶并开盖供居民投放(-2)（1处问题）</t>
+        </is>
+      </c>
+      <c r="G348" s="4" t="inlineStr">
+        <is>
+          <t>查看证据</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>城中村</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>马坑</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="D349" s="6" t="inlineStr">
+        <is>
+          <t>设置消防设施，使用功能正常，取用方便。（2分）</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
+      </c>
+      <c r="F349" s="6" t="inlineStr">
+        <is>
+          <t>（3）其他问题说明（备注描述）(-2)（1处问题）</t>
+        </is>
+      </c>
+      <c r="G349" s="4" t="inlineStr">
+        <is>
+          <t>查看证据</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>城中村</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>马坑</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="D350" s="6" t="inlineStr">
+        <is>
+          <t>各类垃圾及时清运。（2分）</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
+      </c>
+      <c r="F350" s="6" t="inlineStr">
+        <is>
+          <t>（2）暂存点内垃圾清运不及时(-2)（1处问题）</t>
+        </is>
+      </c>
+      <c r="G350" s="4" t="inlineStr">
+        <is>
+          <t>查看证据</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>住宅小区</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>南澳湾花园</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="D351" s="6" t="inlineStr">
+        <is>
+          <t>设置消防设施，使用功能正常，取用方便。（2分）</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
+      </c>
+      <c r="F351" s="6" t="inlineStr">
+        <is>
+          <t>（3）其他问题说明（备注描述）(-2)（1处问题）</t>
+        </is>
+      </c>
+      <c r="G351" s="4" t="inlineStr">
+        <is>
+          <t>查看证据</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>住宅小区</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>南澳湾花园</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="D352" s="6" t="inlineStr">
+        <is>
+          <t>各类垃圾及时清运。（2分）</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
+      </c>
+      <c r="F352" s="6" t="inlineStr">
+        <is>
+          <t>（2）暂存点内垃圾清运不及时(-2)（1处问题）</t>
+        </is>
+      </c>
+      <c r="G352" s="4" t="inlineStr">
+        <is>
+          <t>查看证据</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>城中村</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>老街</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>1.17</t>
+        </is>
+      </c>
+      <c r="D353" s="6" t="inlineStr">
+        <is>
+          <t>转运桶应在黄线划定区域内摆放整齐并保持全天关闭（作业状态除外），禁止罩外摆桶供居民投放。（6分）</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
+      </c>
+      <c r="F353" s="6" t="inlineStr">
+        <is>
+          <t>（3）监控范围外罩外摆桶并开盖供居民投放(-2)（1处问题）</t>
+        </is>
+      </c>
+      <c r="G353" s="4" t="inlineStr">
+        <is>
+          <t>查看证据</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>城中村</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>老街</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="D354" s="6" t="inlineStr">
+        <is>
+          <t>设置消防设施，使用功能正常，取用方便。（2分）</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
+      </c>
+      <c r="F354" s="6" t="inlineStr">
+        <is>
+          <t>（3）其他问题说明（备注描述）(-2)（1处问题）</t>
+        </is>
+      </c>
+      <c r="G354" s="4" t="inlineStr">
+        <is>
+          <t>查看证据</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>城中村</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>老街</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="D355" s="6" t="inlineStr">
+        <is>
+          <t>各类垃圾及时清运。（2分）</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
+      </c>
+      <c r="F355" s="6" t="inlineStr">
+        <is>
+          <t>（2）暂存点内垃圾清运不及时(-2)（1处问题）</t>
+        </is>
+      </c>
+      <c r="G355" s="4" t="inlineStr">
+        <is>
+          <t>查看证据</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>城中村</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>风球山小区</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>1.17</t>
+        </is>
+      </c>
+      <c r="D356" s="6" t="inlineStr">
+        <is>
+          <t>转运桶应在黄线划定区域内摆放整齐并保持全天关闭（作业状态除外），禁止罩外摆桶供居民投放。（6分）</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
+      </c>
+      <c r="F356" s="6" t="inlineStr">
+        <is>
+          <t>（3）监控范围外罩外摆桶并开盖供居民投放(-2)（1处问题）</t>
+        </is>
+      </c>
+      <c r="G356" s="4" t="inlineStr">
+        <is>
+          <t>查看证据</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>城中村</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>风球山小区</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="D357" s="6" t="inlineStr">
+        <is>
+          <t>设置消防设施，使用功能正常，取用方便。（2分）</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
+      </c>
+      <c r="F357" s="6" t="inlineStr">
+        <is>
+          <t>（3）其他问题说明（备注描述）(-2)（1处问题）</t>
+        </is>
+      </c>
+      <c r="G357" s="4" t="inlineStr">
+        <is>
+          <t>查看证据</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>城中村</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>风球山小区</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="D358" s="6" t="inlineStr">
+        <is>
+          <t>各类垃圾及时清运。（2分）</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
+      </c>
+      <c r="F358" s="6" t="inlineStr">
+        <is>
+          <t>（2）暂存点内垃圾清运不及时(-2)（1处问题）</t>
+        </is>
+      </c>
+      <c r="G358" s="4" t="inlineStr">
+        <is>
+          <t>查看证据</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>城中村</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>上企沙</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>1.17</t>
+        </is>
+      </c>
+      <c r="D359" s="6" t="inlineStr">
+        <is>
+          <t>转运桶应在黄线划定区域内摆放整齐并保持全天关闭（作业状态除外），禁止罩外摆桶供居民投放。（6分）</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
+      </c>
+      <c r="F359" s="6" t="inlineStr">
+        <is>
+          <t>（3）监控范围外罩外摆桶并开盖供居民投放(-2)（1处问题）</t>
+        </is>
+      </c>
+      <c r="G359" s="4" t="inlineStr">
+        <is>
+          <t>查看证据</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>住宅小区</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>山海名苑</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>1.17</t>
+        </is>
+      </c>
+      <c r="D360" s="6" t="inlineStr">
+        <is>
+          <t>转运桶应在黄线划定区域内摆放整齐并保持全天关闭（作业状态除外），禁止罩外摆桶供居民投放。（6分）</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>-4</t>
+        </is>
+      </c>
+      <c r="F360" s="6" t="inlineStr">
+        <is>
+          <t>（3）监控范围外罩外摆桶并开盖供居民投放(-2)（2处问题）</t>
+        </is>
+      </c>
+      <c r="G360" s="4" t="inlineStr">
+        <is>
+          <t>查看证据</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>城中村</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>下企沙</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>1.17</t>
+        </is>
+      </c>
+      <c r="D361" s="6" t="inlineStr">
+        <is>
+          <t>转运桶应在黄线划定区域内摆放整齐并保持全天关闭（作业状态除外），禁止罩外摆桶供居民投放。（6分）</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
+      </c>
+      <c r="F361" s="6" t="inlineStr">
+        <is>
+          <t>（3）监控范围外罩外摆桶并开盖供居民投放(-2)（1处问题）</t>
+        </is>
+      </c>
+      <c r="G361" s="4" t="inlineStr">
+        <is>
+          <t>查看证据</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>住宅小区</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>金地朗悦西区</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="D362" s="6" t="inlineStr">
+        <is>
+          <t>分类标志完整、正确、清晰，各类垃圾收集容器外罩和内桶的颜色正确。（4分）</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>-4</t>
+        </is>
+      </c>
+      <c r="F362" s="6" t="inlineStr">
+        <is>
+          <t>（3）外罩和内桶颜色不正确;（不强制要求垃圾桶套袋，若套袋的，收集容器应按垃圾类别对应颜色套袋）(-2)（2处问题）</t>
+        </is>
+      </c>
+      <c r="G362" s="4" t="inlineStr">
+        <is>
+          <t>查看证据</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>住宅小区</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>金地朗悦西区</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>1.13</t>
+        </is>
+      </c>
+      <c r="D363" s="6" t="inlineStr">
+        <is>
+          <t>收集容器外壁及内桶保持干净整洁，避免陈旧性脏污，收集容器内无积水。（4分）</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
+      </c>
+      <c r="F363" s="6" t="inlineStr">
+        <is>
+          <t>（2）收集容器外壁、内桶存在明显陈旧性脏污，大片锈迹等(-2)（1处问题）</t>
+        </is>
+      </c>
+      <c r="G363" s="4" t="inlineStr">
+        <is>
+          <t>查看证据</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>住宅小区</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>金地朗悦西区</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="D364" s="6" t="inlineStr">
+        <is>
+          <t>设置标识牌，外观使用“深i回收”标识，封闭围挡，地面硬底化。（2分）</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
+      </c>
+      <c r="F364" s="6" t="inlineStr">
+        <is>
+          <t>（2）围挡设置不规范（未设置围挡，围挡封闭不全，或使用移动式栅栏、水马等围合）(-2)（1处问题）</t>
+        </is>
+      </c>
+      <c r="G364" s="4" t="inlineStr">
+        <is>
+          <t>查看证据</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>住宅小区</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>金地朗悦东区</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="D365" s="6" t="inlineStr">
+        <is>
+          <t>设置洗手设施。（2分）</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>-1</t>
+        </is>
+      </c>
+      <c r="F365" s="6" t="inlineStr">
+        <is>
+          <t>（3）洗手设施不规范（包括水龙头损坏或明显松动，水龙头不出水，洗手盆堵塞等）(-1)（1处问题）</t>
+        </is>
+      </c>
+      <c r="G365" s="4" t="inlineStr">
+        <is>
+          <t>查看证据</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>住宅小区</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>金地朗悦东区</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="D366" s="6" t="inlineStr">
+        <is>
+          <t>设置标识牌，外观使用“深i回收”标识，封闭围挡，地面硬底化。（2分）</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
+      </c>
+      <c r="F366" s="6" t="inlineStr">
+        <is>
+          <t>（2）围挡设置不规范（未设置围挡，围挡封闭不全，或使用移动式栅栏、水马等围合）(-2)（1处问题）</t>
+        </is>
+      </c>
+      <c r="G366" s="4" t="inlineStr">
         <is>
           <t>查看证据</t>
         </is>
@@ -25013,6 +26409,28 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G342" r:id="rId341"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G343" r:id="rId342"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G344" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G345" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G346" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G347" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G348" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G349" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G350" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G351" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G352" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G353" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G354" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G355" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G356" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G357" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G358" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G359" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G360" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G361" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G362" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G363" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G364" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G365" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G366" r:id="rId365"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>